<commit_message>
[Schematic][BOM] Capacitor added on enable #123
</commit_message>
<xml_diff>
--- a/Design_Files_Reduced_Size/BOM/Client_BOM_Sound_Sensor_v3.2.xlsx
+++ b/Design_Files_Reduced_Size/BOM/Client_BOM_Sound_Sensor_v3.2.xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26529"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\Melih-SoundSensor\Design_Files_Reduced_Size\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Faizan\GitHub\Melih-SoundSensor\Design_Files_Reduced_Size\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28567E1-F201-4D95-98DA-8DE46BA436A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -66,9 +80,6 @@
     <t>C2</t>
   </si>
   <si>
-    <t>C3, C5, C7, C9, C11, C13, C15, C17</t>
-  </si>
-  <si>
     <t>C4, C6, C8, C10, C12, C14, C16, C18</t>
   </si>
   <si>
@@ -421,12 +432,15 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>C3, C5, C7, C9, C11, C13, C15, C17, C48</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1042,26 +1056,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.140625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -1072,34 +1086,34 @@
         <v>12</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>129</v>
-      </c>
       <c r="J1" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K1" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="15">
         <f>ROW(A2) - ROW($A$1)</f>
         <v>1</v>
@@ -1111,22 +1125,22 @@
         <v>13</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J2" s="9">
         <v>6</v>
@@ -1137,7 +1151,7 @@
       </c>
       <c r="L2" s="9"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="17">
         <f t="shared" ref="A3:A25" si="0">ROW(A3) - ROW($A$1)</f>
         <v>2</v>
@@ -1149,22 +1163,22 @@
         <v>14</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J3" s="10">
         <v>1</v>
@@ -1175,7 +1189,7 @@
       </c>
       <c r="L3" s="10"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="15">
         <f>ROW(A4) - ROW($A$1)</f>
         <v>3</v>
@@ -1184,36 +1198,36 @@
         <v>2</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>15</v>
+        <v>133</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J4" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K4" s="9">
         <f>J4*5</f>
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="L4" s="9"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="17">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1222,25 +1236,25 @@
         <v>2</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J5" s="10">
         <v>8</v>
@@ -1251,7 +1265,7 @@
       </c>
       <c r="L5" s="10"/>
     </row>
-    <row r="6" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A6" s="15">
         <f>ROW(A6) - ROW($A$1)</f>
         <v>5</v>
@@ -1260,25 +1274,25 @@
         <v>2</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J6" s="9">
         <v>16</v>
@@ -1289,7 +1303,7 @@
       </c>
       <c r="L6" s="9"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="17">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1298,25 +1312,25 @@
         <v>2</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J7" s="10">
         <v>6</v>
@@ -1327,7 +1341,7 @@
       </c>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="15">
         <f>ROW(A8) - ROW($A$1)</f>
         <v>7</v>
@@ -1336,25 +1350,25 @@
         <v>2</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J8" s="9">
         <v>2</v>
@@ -1365,7 +1379,7 @@
       </c>
       <c r="L8" s="9"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="17">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1374,25 +1388,25 @@
         <v>2</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J9" s="10">
         <v>1</v>
@@ -1403,34 +1417,34 @@
       </c>
       <c r="L9" s="10"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
         <f>ROW(A10) - ROW($A$1)</f>
         <v>9</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1441,7 +1455,7 @@
       </c>
       <c r="L10" s="9"/>
     </row>
-    <row r="11" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A11" s="17">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1450,25 +1464,25 @@
         <v>3</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J11" s="10">
         <v>1</v>
@@ -1479,7 +1493,7 @@
       </c>
       <c r="L11" s="10"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="15">
         <f>ROW(A12) - ROW($A$1)</f>
         <v>11</v>
@@ -1488,25 +1502,25 @@
         <v>4</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>
@@ -1517,7 +1531,7 @@
       </c>
       <c r="L12" s="9"/>
     </row>
-    <row r="13" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A13" s="17">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1526,25 +1540,25 @@
         <v>5</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J13" s="10">
         <v>1</v>
@@ -1555,7 +1569,7 @@
       </c>
       <c r="L13" s="10"/>
     </row>
-    <row r="14" spans="1:12" ht="36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A14" s="15">
         <f>ROW(A14) - ROW($A$1)</f>
         <v>13</v>
@@ -1564,25 +1578,25 @@
         <v>6</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1593,7 +1607,7 @@
       </c>
       <c r="L14" s="9"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="17">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1602,25 +1616,25 @@
         <v>7</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J15" s="10">
         <v>8</v>
@@ -1631,7 +1645,7 @@
       </c>
       <c r="L15" s="10"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="15">
         <f>ROW(A16) - ROW($A$1)</f>
         <v>15</v>
@@ -1640,25 +1654,25 @@
         <v>8</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
@@ -1669,7 +1683,7 @@
       </c>
       <c r="L16" s="9"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1678,25 +1692,25 @@
         <v>8</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J17" s="10">
         <v>3</v>
@@ -1707,7 +1721,7 @@
       </c>
       <c r="L17" s="10"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="15">
         <f>ROW(A18) - ROW($A$1)</f>
         <v>17</v>
@@ -1716,25 +1730,25 @@
         <v>8</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1745,7 +1759,7 @@
       </c>
       <c r="L18" s="9"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="17">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1754,25 +1768,25 @@
         <v>8</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J19" s="10">
         <v>2</v>
@@ -1783,7 +1797,7 @@
       </c>
       <c r="L19" s="10"/>
     </row>
-    <row r="20" spans="1:12" ht="36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A20" s="15">
         <f>ROW(A20) - ROW($A$1)</f>
         <v>19</v>
@@ -1792,25 +1806,25 @@
         <v>9</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I20" s="26" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1821,7 +1835,7 @@
       </c>
       <c r="L20" s="9"/>
     </row>
-    <row r="21" spans="1:12" ht="36" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A21" s="17">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1830,25 +1844,25 @@
         <v>9</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J21" s="10">
         <v>1</v>
@@ -1859,7 +1873,7 @@
       </c>
       <c r="L21" s="10"/>
     </row>
-    <row r="22" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A22" s="15">
         <f>ROW(A22) - ROW($A$1)</f>
         <v>21</v>
@@ -1868,25 +1882,25 @@
         <v>10</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -1897,7 +1911,7 @@
       </c>
       <c r="L22" s="9"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="17">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -1906,25 +1920,25 @@
         <v>10</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J23" s="10">
         <v>1</v>
@@ -1935,7 +1949,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="15">
         <f>ROW(A24) - ROW($A$1)</f>
         <v>23</v>
@@ -1944,25 +1958,25 @@
         <v>11</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -1973,34 +1987,34 @@
       </c>
       <c r="L24" s="9"/>
     </row>
-    <row r="25" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="17">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="I25" s="26" t="s">
         <v>130</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="I25" s="26" t="s">
-        <v>131</v>
       </c>
       <c r="J25" s="10">
         <v>1</v>
@@ -2011,7 +2025,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="19"/>
       <c r="B26" s="20"/>
       <c r="C26" s="21"/>
@@ -2025,7 +2039,7 @@
       <c r="K26" s="8"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
       <c r="B27" s="13"/>
       <c r="C27" s="1"/>

</xml_diff>